<commit_message>
Timetable Template from Bulk Import to get the new file.
</commit_message>
<xml_diff>
--- a/backend/format/Timetable_Bulk_Import_Template.xlsx
+++ b/backend/format/Timetable_Bulk_Import_Template.xlsx
@@ -399,6 +399,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I4"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,13 +425,13 @@
         <v>Session</v>
       </c>
       <c r="E1" t="str">
+        <v>Department</v>
+      </c>
+      <c r="F1" t="str">
         <v>Course Code</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Course Name</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Department</v>
       </c>
       <c r="H1" t="str">
         <v>Batch</v>
@@ -431,7 +442,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-16</v>
       </c>
       <c r="B2" t="str">
         <v>09:00</v>
@@ -443,16 +454,16 @@
         <v>FN</v>
       </c>
       <c r="E2" t="str">
-        <v>24BCS101</v>
+        <v>BCS</v>
       </c>
       <c r="F2" t="str">
-        <v>Data Structures</v>
+        <v>24BCS102</v>
       </c>
       <c r="G2" t="str">
-        <v>BCS</v>
+        <v>Database Management Systems</v>
       </c>
       <c r="H2" t="str">
-        <v>24BCS</v>
+        <v>2024-2028</v>
       </c>
       <c r="I2" t="str">
         <v>CAT1</v>
@@ -460,7 +471,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-16</v>
       </c>
       <c r="B3" t="str">
         <v>14:00</v>
@@ -472,16 +483,16 @@
         <v>AN</v>
       </c>
       <c r="E3" t="str">
-        <v>24BAD201</v>
+        <v>BCS</v>
       </c>
       <c r="F3" t="str">
-        <v>Database Management</v>
+        <v>24BCS101</v>
       </c>
       <c r="G3" t="str">
-        <v>BAD</v>
+        <v>Data Structures</v>
       </c>
       <c r="H3" t="str">
-        <v>24BAD</v>
+        <v>2024-2028</v>
       </c>
       <c r="I3" t="str">
         <v>CAT1</v>
@@ -489,7 +500,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-09-30</v>
+        <v>2026-10-17</v>
       </c>
       <c r="B4" t="str">
         <v>09:00</v>
@@ -501,16 +512,16 @@
         <v>FN</v>
       </c>
       <c r="E4" t="str">
-        <v>24BIT301</v>
+        <v>BAD</v>
       </c>
       <c r="F4" t="str">
-        <v>Computer Networks</v>
+        <v>24BAD201</v>
       </c>
       <c r="G4" t="str">
-        <v>BIT</v>
+        <v>Database Management</v>
       </c>
       <c r="H4" t="str">
-        <v>24BIT</v>
+        <v>2023-2027</v>
       </c>
       <c r="I4" t="str">
         <v>CAT2</v>
@@ -525,7 +536,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A43"/>
+  <cols>
+    <col min="1" max="1" width="100.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -539,7 +553,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>INSTRUCTIONS:</v>
+        <v>Matches Timetable → Add Schedule fields.</v>
       </c>
     </row>
     <row r="4">
@@ -549,22 +563,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>1. Fill in the "Timetable" sheet with your exam schedule data</v>
+        <v>INSTRUCTIONS:</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2. Follow the exact format shown in the sample rows</v>
+        <v>1. Fill the "Timetable" sheet. Keep the header row exactly as given.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>3. Delete the sample data before importing (or keep as reference)</v>
+        <v>2. Replace sample rows with your real schedules (or delete samples).</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>4. Save the file and upload via the Bulk Import tab</v>
+        <v>3. Save as .xlsx and upload via Bulk Import.</v>
       </c>
     </row>
     <row r="9">
@@ -579,7 +593,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Date | Start Time | End Time | Session | Course Code | Course Name | Department | Batch | Exam Type</v>
+        <v>Date | Start Time | End Time | Session | Department | Course Code | Course Name | Batch | Exam Type</v>
       </c>
     </row>
     <row r="12">
@@ -594,7 +608,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">  • Format: YYYY-MM-DD (e.g., 2026-09-29)</v>
+        <v xml:space="preserve">  • Format: YYYY-MM-DD (e.g. 2026-10-20)</v>
       </c>
     </row>
     <row r="15">
@@ -614,7 +628,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">  • Format: HH:MM in 24-hour format (e.g., 09:00, 14:00)</v>
+        <v xml:space="preserve">  • Format: HH:MM in 24-hour (e.g. 09:00, 14:00)</v>
       </c>
     </row>
     <row r="19">
@@ -634,87 +648,117 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  • Only FN or AN (case-sensitive uppercase)</v>
+        <v xml:space="preserve">  • FN or AN only (uppercase)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v/>
+        <v xml:space="preserve">  • FN → morning start; AN → afternoon start</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Course Code / Course Name:</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  • Course Code must exist in student data for the Department/Batch</v>
+        <v>Department:</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v/>
+        <v xml:space="preserve">  • Uppercase department code (e.g. BCS, BAD, BIT)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Department:</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  • Uppercase 3-letter code (e.g., BCS, BAD, BIT, BCE, BME)</v>
+        <v>Course Code / Course Name:</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v xml:space="preserve">  • Same values as Add Schedule dropdown / auto-filled name</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Batch (REQUIRED):</v>
+        <v xml:space="preserve">  • Course must be enrolled by students in that Department + Batch</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  • Format: YY + Department Code — pattern ^[0-9]{2}[A-Z]{3}$</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  • Examples: 24BCS, 24BAD, 24BIT</v>
+        <v>Batch (REQUIRED):</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  • Must match Department (Department=BCS → Batch like 24BCS)</v>
+        <v xml:space="preserve">  • Use the Batch Management batch name (e.g. 2024-2028, 2023-2027)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  • Batch must already exist in the Academic Context (not auto-created)</v>
+        <v xml:space="preserve">  • Same Batch shown in Add Schedule after selecting Course</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v xml:space="preserve">  • Batch must already exist in the selected Academic Context</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Exam Type:</v>
+        <v xml:space="preserve">  • Do NOT invent register-number prefixes as batches (e.g. do not use 24BCS unless that is a real Batch name)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  • Only CAT1, CAT2, or SEM (case-sensitive uppercase)</v>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Exam Type:</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v xml:space="preserve">  • CAT1, CAT2, or SEM (uppercase, no spaces)</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v xml:space="preserve">  • Same as Add Schedule: CAT 1 → CAT1, CAT 2 → CAT2, Semester → SEM</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Students:</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">  • Not entered in Excel. Loaded automatically from Course + Batch enrollments (same as Add Schedule).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CAT 1 / CAT1 / CAT-1 / SA 1 / SA-1 → SA1
</commit_message>
<xml_diff>
--- a/backend/format/Timetable_Bulk_Import_Template.xlsx
+++ b/backend/format/Timetable_Bulk_Import_Template.xlsx
@@ -442,7 +442,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-10-16</v>
+        <v>2026-11-05</v>
       </c>
       <c r="B2" t="str">
         <v>09:00</v>
@@ -466,12 +466,12 @@
         <v>2024-2028</v>
       </c>
       <c r="I2" t="str">
-        <v>CAT1</v>
+        <v>SA1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-10-16</v>
+        <v>2026-11-05</v>
       </c>
       <c r="B3" t="str">
         <v>14:00</v>
@@ -495,12 +495,12 @@
         <v>2024-2028</v>
       </c>
       <c r="I3" t="str">
-        <v>CAT1</v>
+        <v>SA1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-10-17</v>
+        <v>2026-11-06</v>
       </c>
       <c r="B4" t="str">
         <v>09:00</v>
@@ -524,7 +524,7 @@
         <v>2023-2027</v>
       </c>
       <c r="I4" t="str">
-        <v>CAT2</v>
+        <v>SA2</v>
       </c>
     </row>
   </sheetData>
@@ -536,7 +536,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A45"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
@@ -733,32 +733,42 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">  • CAT1, CAT2, or SEM (uppercase, no spaces)</v>
+        <v xml:space="preserve">  • SA1, SA2, or SEM (preferred storage values)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">  • Same as Add Schedule: CAT 1 → CAT1, CAT 2 → CAT2, Semester → SEM</v>
+        <v xml:space="preserve">  • CAT 1 / CAT1 / CAT-1 are accepted and stored as SA1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v/>
+        <v xml:space="preserve">  • CAT 2 / CAT2 / CAT-2 are accepted and stored as SA2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Students:</v>
+        <v xml:space="preserve">  • SA 1 / SA-1 → SA1; SA 2 / SA-2 → SA2; Semester → SEM</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Students:</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
         <v xml:space="preserve">  • Not entered in Excel. Loaded automatically from Course + Batch enrollments (same as Add Schedule).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>